<commit_message>
Cleanup: 105 test/debug dosya silindi - sistem optimize edildi
</commit_message>
<xml_diff>
--- a/data/belgrad/service_status.xlsx
+++ b/data/belgrad/service_status.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H27"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1284,8 +1284,6 @@
           <t>Servis</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>Toplu servise alındı</t>
@@ -1297,6 +1295,808 @@
         </is>
       </c>
       <c r="H27" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>1531</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:19</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1532</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:20</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>1533</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:20</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>1534</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:20</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>1535</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:20</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1536</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:20</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>1537</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:20</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>1538</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:20</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1539</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:20</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>1540</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:20</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1541</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:20</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>1542</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:20</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>1543</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:21</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>1544</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:21</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>1545</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:21</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>1546</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:21</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>1547</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:21</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>1548</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:21</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>1549</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:21</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>1550</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:21</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>1551</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:22</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>1552</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:22</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>1553</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:22</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>1554</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:22</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>1555</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2026-03-02 09:21:22</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
         <is>
           <t>admin</t>
         </is>

</xml_diff>

<commit_message>
SSHv2.0 - Excel not sistemi, beyaz bold font, border, availability fix, tarih siralama
</commit_message>
<xml_diff>
--- a/data/belgrad/service_status.xlsx
+++ b/data/belgrad/service_status.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3780,8 +3780,6 @@
           <t>Servis</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr"/>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>Toplu servise alındı</t>
@@ -3793,6 +3791,808 @@
         </is>
       </c>
       <c r="H105" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>1531</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:16</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1532</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:16</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>1533</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:17</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>1534</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:17</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>1535</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:17</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1536</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:17</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>1537</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:17</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>1538</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:18</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1539</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:18</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>1540</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:18</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>1541</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:18</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1542</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:19</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1543</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:19</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>1544</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:19</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>1545</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:19</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>1546</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:19</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>1547</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:20</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>1548</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:20</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>1549</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:20</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>1550</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:20</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>1551</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:21</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>1552</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:21</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1553</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:21</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>1554</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:21</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2026-04-09</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>1555</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Servis</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>Toplu servise alındı</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>2026-04-09 00:26:21</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
         <is>
           <t>admin</t>
         </is>

</xml_diff>